<commit_message>
CreateEntity refactor, wizard & blacksmith additions, many fixes.
</commit_message>
<xml_diff>
--- a/Other/RoStatProcessing.xlsx
+++ b/Other/RoStatProcessing.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\ProjectsSSD\RagnarokRebuildTcp\Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B954FCCB-58D8-4CD1-87E2-1FC3CF582267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0418A210-368A-4AD8-88DA-462608D61300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="497" yWindow="2606" windowWidth="31080" windowHeight="14828" firstSheet="3" activeTab="7" xr2:uid="{1C41742B-2950-4FF8-AA39-6557869B44EA}"/>
+    <workbookView xWindow="4946" yWindow="3463" windowWidth="23725" windowHeight="12643" xr2:uid="{1C41742B-2950-4FF8-AA39-6557869B44EA}"/>
   </bookViews>
   <sheets>
     <sheet name="StatDef" sheetId="3" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3328" uniqueCount="1236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3337" uniqueCount="1239">
   <si>
     <t>Id</t>
   </si>
@@ -3761,6 +3761,15 @@
   </si>
   <si>
     <t>SecondJob</t>
+  </si>
+  <si>
+    <t>FUBUKI</t>
+  </si>
+  <si>
+    <t>Fubuki</t>
+  </si>
+  <si>
+    <t>fubuki.asset</t>
   </si>
 </sst>
 </file>
@@ -4211,7 +4220,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{811A97A5-94A7-4FFA-A162-65D076B52481}">
-  <dimension ref="A1:AK325"/>
+  <dimension ref="A1:AK326"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="5.07421875" bestFit="1" customWidth="1"/>
@@ -39346,6 +39355,113 @@
         <v>1</v>
       </c>
     </row>
+    <row r="326" spans="1:36" x14ac:dyDescent="0.4">
+      <c r="A326">
+        <v>6022</v>
+      </c>
+      <c r="B326" t="s">
+        <v>1236</v>
+      </c>
+      <c r="C326" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D326">
+        <v>62</v>
+      </c>
+      <c r="E326">
+        <v>60</v>
+      </c>
+      <c r="F326">
+        <v>100</v>
+      </c>
+      <c r="G326">
+        <v>10</v>
+      </c>
+      <c r="H326">
+        <v>30</v>
+      </c>
+      <c r="I326">
+        <v>130</v>
+      </c>
+      <c r="J326">
+        <v>100</v>
+      </c>
+      <c r="K326">
+        <v>100</v>
+      </c>
+      <c r="L326">
+        <v>80</v>
+      </c>
+      <c r="M326">
+        <v>15</v>
+      </c>
+      <c r="N326">
+        <v>9</v>
+      </c>
+      <c r="O326">
+        <v>120</v>
+      </c>
+      <c r="P326">
+        <v>30</v>
+      </c>
+      <c r="Q326">
+        <v>90</v>
+      </c>
+      <c r="R326">
+        <v>90</v>
+      </c>
+      <c r="S326">
+        <v>10</v>
+      </c>
+      <c r="T326">
+        <v>12</v>
+      </c>
+      <c r="U326" t="s">
+        <v>38</v>
+      </c>
+      <c r="V326" t="s">
+        <v>160</v>
+      </c>
+      <c r="W326" t="s">
+        <v>532</v>
+      </c>
+      <c r="X326">
+        <v>1000</v>
+      </c>
+      <c r="Y326">
+        <v>750</v>
+      </c>
+      <c r="Z326">
+        <v>1000</v>
+      </c>
+      <c r="AA326">
+        <v>160</v>
+      </c>
+      <c r="AB326" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC326" t="s">
+        <v>1112</v>
+      </c>
+      <c r="AD326" t="s">
+        <v>99</v>
+      </c>
+      <c r="AF326">
+        <v>972</v>
+      </c>
+      <c r="AG326" t="s">
+        <v>1238</v>
+      </c>
+      <c r="AH326">
+        <v>0</v>
+      </c>
+      <c r="AI326">
+        <v>0.5</v>
+      </c>
+      <c r="AJ326">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:AJ180">
     <sortCondition ref="D3:D180"/>
@@ -65604,7 +65720,7 @@
         <v>1060506</v>
       </c>
       <c r="E67">
-        <f t="shared" ref="E67:E70" si="2">(C68/C67-1)*(1-(A67/500))+1</f>
+        <f t="shared" ref="E67:E69" si="2">(C68/C67-1)*(1-(A67/500))+1</f>
         <v>1.0718704844668487</v>
       </c>
       <c r="F67">

</xml_diff>

<commit_message>
Map processing adustments, monster sleeping, config options, teleport fixes, feature flags, and more.
</commit_message>
<xml_diff>
--- a/Other/RoStatProcessing.xlsx
+++ b/Other/RoStatProcessing.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\ProjectsSSD\RagnarokRebuildTcp\Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD1BC145-16DC-4AFC-B66F-F14CB919AEDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F19434F6-8650-4998-8E08-8F2300D5F2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5486" yWindow="1586" windowWidth="24034" windowHeight="14691" xr2:uid="{1C41742B-2950-4FF8-AA39-6557869B44EA}"/>
+    <workbookView xWindow="5631" yWindow="4149" windowWidth="26323" windowHeight="12642" xr2:uid="{1C41742B-2950-4FF8-AA39-6557869B44EA}"/>
   </bookViews>
   <sheets>
     <sheet name="StatDef" sheetId="3" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3438" uniqueCount="1276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3452" uniqueCount="1278">
   <si>
     <t>Id</t>
   </si>
@@ -3881,6 +3881,12 @@
   </si>
   <si>
     <t>Gig</t>
+  </si>
+  <si>
+    <t>DoddlerCustomMobs</t>
+  </si>
+  <si>
+    <t>Feature</t>
   </si>
 </sst>
 </file>
@@ -3986,12 +3992,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5AE4419D-5DB5-4D1B-9713-9E17C7E1903B}" name="Table1" displayName="Table1" ref="A1:AK425" totalsRowShown="0">
-  <autoFilter ref="A1:AK425" xr:uid="{5AE4419D-5DB5-4D1B-9713-9E17C7E1903B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5AE4419D-5DB5-4D1B-9713-9E17C7E1903B}" name="Table1" displayName="Table1" ref="A1:AL425" totalsRowShown="0">
+  <autoFilter ref="A1:AL425" xr:uid="{5AE4419D-5DB5-4D1B-9713-9E17C7E1903B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AK331">
     <sortCondition ref="A1:A425"/>
   </sortState>
-  <tableColumns count="37">
+  <tableColumns count="38">
     <tableColumn id="1" xr3:uid="{B859DFBF-EB68-4198-9FF0-FEBC6A5D6D92}" name="Id"/>
     <tableColumn id="2" xr3:uid="{A79D65AB-A01E-4B86-B9DF-A89CDC4EC4AA}" name="Code"/>
     <tableColumn id="3" xr3:uid="{EE52CDA5-01D0-433C-8F91-38DC3D87119D}" name="Name"/>
@@ -4029,6 +4035,7 @@
     <tableColumn id="34" xr3:uid="{C2F7284A-9A1E-41FB-B9B4-55E9E8237CF0}" name="ClientShadow"/>
     <tableColumn id="35" xr3:uid="{4A5E8A7E-1FED-40FB-B528-9E07702DC74A}" name="ClientSize"/>
     <tableColumn id="36" xr3:uid="{A1CBDEC4-7472-419D-A040-958DE222AA8B}" name="Flags"/>
+    <tableColumn id="38" xr3:uid="{6BCAD2AE-AAFA-4CFC-AC03-A9C328911CC9}" name="Feature"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4331,7 +4338,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{811A97A5-94A7-4FFA-A162-65D076B52481}">
-  <dimension ref="A1:AK337"/>
+  <dimension ref="A1:AL337"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="5.07421875" bestFit="1" customWidth="1"/>
@@ -4368,9 +4375,10 @@
     <col min="35" max="35" width="14.84375" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="11.3828125" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="36.3046875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="21.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4482,8 +4490,11 @@
       <c r="AK1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL1" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>3999</v>
       </c>
@@ -4590,7 +4601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>4000</v>
       </c>
@@ -4697,7 +4708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>4001</v>
       </c>
@@ -4804,7 +4815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>4002</v>
       </c>
@@ -4911,7 +4922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>4003</v>
       </c>
@@ -5018,7 +5029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>4004</v>
       </c>
@@ -5128,7 +5139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>4005</v>
       </c>
@@ -5235,7 +5246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>4006</v>
       </c>
@@ -5342,7 +5353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>4007</v>
       </c>
@@ -5449,7 +5460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>4008</v>
       </c>
@@ -5556,7 +5567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>4009</v>
       </c>
@@ -5666,7 +5677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>4010</v>
       </c>
@@ -5773,7 +5784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>4011</v>
       </c>
@@ -5883,7 +5894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>4012</v>
       </c>
@@ -5990,7 +6001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>4013</v>
       </c>
@@ -37180,7 +37191,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="305" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="305" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A305">
         <v>4302</v>
       </c>
@@ -37287,7 +37298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="306" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A306">
         <v>4303</v>
       </c>
@@ -37394,7 +37405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="307" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="307" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A307">
         <v>4304</v>
       </c>
@@ -37501,7 +37512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="308" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="308" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A308">
         <v>4305</v>
       </c>
@@ -37608,7 +37619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="309" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="309" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A309">
         <v>4306</v>
       </c>
@@ -37718,7 +37729,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="310" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="310" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A310">
         <v>4307</v>
       </c>
@@ -37828,7 +37839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="311" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="311" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A311">
         <v>4308</v>
       </c>
@@ -37935,7 +37946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="312" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="312" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A312">
         <v>4309</v>
       </c>
@@ -38042,7 +38053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="313" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="313" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A313">
         <v>4310</v>
       </c>
@@ -38149,7 +38160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="314" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="314" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A314">
         <v>4311</v>
       </c>
@@ -38256,7 +38267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="315" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A315">
         <v>4312</v>
       </c>
@@ -38363,7 +38374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="316" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="316" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A316">
         <v>5000</v>
       </c>
@@ -38470,7 +38481,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="317" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="317" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A317">
         <v>6000</v>
       </c>
@@ -38580,7 +38591,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="318" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="318" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A318">
         <v>6001</v>
       </c>
@@ -38687,7 +38698,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="319" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="319" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A319">
         <v>6002</v>
       </c>
@@ -38797,7 +38808,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="320" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="320" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A320">
         <v>6003</v>
       </c>
@@ -38906,8 +38917,11 @@
       <c r="AJ320">
         <v>1</v>
       </c>
-    </row>
-    <row r="321" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL320" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="321" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A321">
         <v>6004</v>
       </c>
@@ -39013,8 +39027,11 @@
       <c r="AJ321">
         <v>1</v>
       </c>
-    </row>
-    <row r="322" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL321" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="322" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A322">
         <v>6005</v>
       </c>
@@ -39123,8 +39140,11 @@
       <c r="AK322" t="s">
         <v>1130</v>
       </c>
-    </row>
-    <row r="323" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL322" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="323" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A323">
         <v>6006</v>
       </c>
@@ -39233,8 +39253,11 @@
       <c r="AJ323">
         <v>1</v>
       </c>
-    </row>
-    <row r="324" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL323" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="324" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A324">
         <v>6007</v>
       </c>
@@ -39343,8 +39366,11 @@
       <c r="AJ324">
         <v>1</v>
       </c>
-    </row>
-    <row r="325" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL324" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="325" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A325">
         <v>6008</v>
       </c>
@@ -39453,8 +39479,11 @@
       <c r="AJ325">
         <v>1</v>
       </c>
-    </row>
-    <row r="326" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL325" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="326" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A326">
         <v>6009</v>
       </c>
@@ -39563,8 +39592,11 @@
       <c r="AJ326">
         <v>1</v>
       </c>
-    </row>
-    <row r="327" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL326" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="327" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A327">
         <v>6010</v>
       </c>
@@ -39673,8 +39705,11 @@
       <c r="AJ327">
         <v>1</v>
       </c>
-    </row>
-    <row r="328" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL327" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="328" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A328">
         <v>6011</v>
       </c>
@@ -39783,8 +39818,11 @@
       <c r="AJ328">
         <v>1</v>
       </c>
-    </row>
-    <row r="329" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL328" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="329" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A329">
         <v>6012</v>
       </c>
@@ -39893,8 +39931,11 @@
       <c r="AJ329">
         <v>1.05</v>
       </c>
-    </row>
-    <row r="330" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL329" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="330" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A330">
         <v>6013</v>
       </c>
@@ -40003,8 +40044,11 @@
       <c r="AJ330">
         <v>1</v>
       </c>
-    </row>
-    <row r="331" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL330" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="331" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A331">
         <v>6014</v>
       </c>
@@ -40113,8 +40157,11 @@
       <c r="AJ331">
         <v>1</v>
       </c>
-    </row>
-    <row r="332" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="AL331" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="332" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A332">
         <v>6015</v>
       </c>
@@ -40221,7 +40268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="333" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="333" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A333">
         <v>6018</v>
       </c>
@@ -40328,7 +40375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="334" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="334" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A334">
         <v>6019</v>
       </c>
@@ -40435,7 +40482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="335" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="335" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A335">
         <v>6020</v>
       </c>
@@ -40542,7 +40589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="336" spans="1:37" x14ac:dyDescent="0.4">
+    <row r="336" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A336">
         <v>6021</v>
       </c>
@@ -40649,7 +40696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="337" spans="1:36" x14ac:dyDescent="0.4">
+    <row r="337" spans="1:38" x14ac:dyDescent="0.4">
       <c r="A337">
         <v>6022</v>
       </c>
@@ -40754,6 +40801,9 @@
       </c>
       <c r="AJ337">
         <v>1</v>
+      </c>
+      <c r="AL337" t="s">
+        <v>1276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>